<commit_message>
Separar sección de importar de app
</commit_message>
<xml_diff>
--- a/data/ArchivosLimpios/new_distribuidor.xlsx
+++ b/data/ArchivosLimpios/new_distribuidor.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,11 +460,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>IAFSA - JJAM0280</t>
+          <t>IAFSA - 4100035M</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -474,12 +474,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>CASE IH</t>
+          <t>NEW HOLLAND AG</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Magnum 290</t>
+          <t>TS6.120 ELITE</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -493,16 +493,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>1216.46</v>
+        <v>1104.18</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>IAFSA - 4100035M</t>
+          <t>IAFSA - NKJ0B80CTNKH30828</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -512,35 +512,35 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NEW HOLLAND AG</t>
+          <t>NEW HOLLAND CE</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>TS6.120 ELITE</t>
+          <t>B80C</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Tamaulipas</t>
+          <t>Nuevo León</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Valle Hermoso</t>
+          <t>Galeana</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1104.18</v>
+        <v>454.09</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CTNKH30831</t>
+          <t>IAFSA - NKJ0B80CKNKH30816</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -569,16 +569,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>478.42</v>
+        <v>247.41</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CTNKH30828</t>
+          <t>IAFSA - NKJ0B80CKNKH30816</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -603,20 +603,20 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Galeana</t>
+          <t>Lampazos de Naranjo</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>454.09</v>
+        <v>194.98</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CKNKH30816</t>
+          <t>IAFSA - NKJ0B80CHNKH30825</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -641,20 +641,20 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Guadalupe</t>
+          <t>San Nicolás de los Garza</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>420.73</v>
+        <v>51.77</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CKPKH34433</t>
+          <t>IAFSA - NKJ0B80CTNKH30831</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -679,20 +679,20 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>General Escobedo</t>
+          <t>Cadereyta Jiménez</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>330.45</v>
+        <v>34.41</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CKNKH30816</t>
+          <t>IAFSA - NKJ0B80CHNKH30825</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -717,20 +717,20 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>General Escobedo</t>
+          <t>Ciudad Santa Catarina</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>247.41</v>
+        <v>23.23</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CKNKH30816</t>
+          <t>IAFSA - NKJ0B80CTNKH30831</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -755,20 +755,20 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Lampazos de Naranjo</t>
+          <t>Apodaca</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>194.98</v>
+        <v>18.59</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CKPKH34433</t>
+          <t>IAFSA - NKJ0B80CTNKH30831</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -788,21 +788,21 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Nuevo León</t>
+          <t>Chihuahua</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Apodaca</t>
+          <t>Chihuahua</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>189.04</v>
+        <v>9.31</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -831,20 +831,20 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Monterrey</t>
+          <t>El Carmen</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>185.97</v>
+        <v>3.57</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CKPKH34433</t>
+          <t>IAFSA - NKJ0B80CHNKH30825</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -869,20 +869,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Monterrey</t>
+          <t>Guadalupe</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>170.86</v>
+        <v>3.07</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CKPKH34433</t>
+          <t>IAFSA - NKJ0B80CHNKH30825</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -907,20 +907,20 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Cadereyta Jiménez</t>
+          <t>Monterrey</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>170.2</v>
+        <v>0.51</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CKPKH34433</t>
+          <t>IAFSA - NKJ0B80CHNKH30825</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -949,614 +949,6 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>145.79</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>IAFSA - NKJ0B80CKNKH30816</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>NEW HOLLAND CE</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>B80C</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Nuevo León</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>San Pedro Garza García</t>
-        </is>
-      </c>
-      <c r="H15" t="n">
-        <v>138.63</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>IAFSA - NKJ0B80CTNKH30831</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>NEW HOLLAND CE</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>B80C</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Nuevo León</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>San Nicolás de los Garza</t>
-        </is>
-      </c>
-      <c r="H16" t="n">
-        <v>136.8</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>IAFSA - NKJ0B80CTNKH30831</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>NEW HOLLAND CE</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>B80C</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Nuevo León</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>San Pedro Garza García</t>
-        </is>
-      </c>
-      <c r="H17" t="n">
-        <v>108.41</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>IAFSA - NKJ0B80CKNKH30816</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>NEW HOLLAND CE</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>B80C</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Nuevo León</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Ciudad Santa Catarina</t>
-        </is>
-      </c>
-      <c r="H18" t="n">
-        <v>87.22</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>IAFSA - NKJ0B80CKPKH34433</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>NEW HOLLAND CE</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>B80C</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Nuevo León</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Guadalupe</t>
-        </is>
-      </c>
-      <c r="H19" t="n">
-        <v>64.38</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>IAFSA - NKJ0B80CTNKH30831</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>NEW HOLLAND CE</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>B80C</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Nuevo León</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Guadalupe</t>
-        </is>
-      </c>
-      <c r="H20" t="n">
-        <v>62.04</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>IAFSA - NKJ0B80CKPKH34433</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>NEW HOLLAND CE</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>B80C</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Nuevo León</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Ciudad Santa Catarina</t>
-        </is>
-      </c>
-      <c r="H21" t="n">
-        <v>58.98</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>IAFSA - NKJ0B80CHNKH30825</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>NEW HOLLAND CE</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>B80C</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Nuevo León</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>San Nicolás de los Garza</t>
-        </is>
-      </c>
-      <c r="H22" t="n">
-        <v>51.77</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>IAFSA - NKJ0B80CTNKH30831</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>NEW HOLLAND CE</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>B80C</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Nuevo León</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Cadereyta Jiménez</t>
-        </is>
-      </c>
-      <c r="H23" t="n">
-        <v>34.41</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>IAFSA - NKJ0B80CHNKH30825</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>NEW HOLLAND CE</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>B80C</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Nuevo León</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Ciudad Santa Catarina</t>
-        </is>
-      </c>
-      <c r="H24" t="n">
-        <v>23.23</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>IAFSA - NKJ0B80CTNKH30831</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>NEW HOLLAND CE</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>B80C</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Nuevo León</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Apodaca</t>
-        </is>
-      </c>
-      <c r="H25" t="n">
-        <v>18.59</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>IAFSA - NKJ0B80CTNKH30831</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>NEW HOLLAND CE</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>B80C</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Chihuahua</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Chihuahua</t>
-        </is>
-      </c>
-      <c r="H26" t="n">
-        <v>9.31</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>IAFSA - NKJ0B80CTNKH30831</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>NEW HOLLAND CE</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>B80C</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Nuevo León</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>El Carmen</t>
-        </is>
-      </c>
-      <c r="H27" t="n">
-        <v>3.57</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>IAFSA - NKJ0B80CHNKH30825</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>NEW HOLLAND CE</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>B80C</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Nuevo León</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Guadalupe</t>
-        </is>
-      </c>
-      <c r="H28" t="n">
-        <v>3.07</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>IAFSA - NKJ0B80CHNKH30825</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>NEW HOLLAND CE</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>B80C</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Nuevo León</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Monterrey</t>
-        </is>
-      </c>
-      <c r="H29" t="n">
-        <v>0.51</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>IAFSA - NKJ0B80CHNKH30825</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>NEW HOLLAND CE</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>B80C</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Nuevo León</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>San Pedro Garza García</t>
-        </is>
-      </c>
-      <c r="H30" t="n">
         <v>0.04</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar orden de gráficos y espacios
</commit_message>
<xml_diff>
--- a/data/ArchivosLimpios/new_distribuidor.xlsx
+++ b/data/ArchivosLimpios/new_distribuidor.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,11 +460,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>IAFSA - 4100035M</t>
+          <t>IAFSA - JJAM0280</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -474,12 +474,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NEW HOLLAND AG</t>
+          <t>CASE IH</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>TS6.120 ELITE</t>
+          <t>Magnum 290</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -493,16 +493,16 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>1104.18</v>
+        <v>1216.46</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CTNKH30828</t>
+          <t>IAFSA - 4100035M</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -512,35 +512,35 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NEW HOLLAND CE</t>
+          <t>NEW HOLLAND AG</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>B80C</t>
+          <t>TS6.120 ELITE</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Nuevo León</t>
+          <t>Tamaulipas</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Galeana</t>
+          <t>Valle Hermoso</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>454.09</v>
+        <v>1104.18</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CKNKH30816</t>
+          <t>IAFSA - NKJ0B80CTNKH30831</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -569,16 +569,16 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>247.41</v>
+        <v>478.42</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CKNKH30816</t>
+          <t>IAFSA - NKJ0B80CTNKH30828</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -603,20 +603,20 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Lampazos de Naranjo</t>
+          <t>Galeana</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>194.98</v>
+        <v>454.09</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CHNKH30825</t>
+          <t>IAFSA - NKJ0B80CKNKH30816</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -641,20 +641,20 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>San Nicolás de los Garza</t>
+          <t>Guadalupe</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>51.77</v>
+        <v>420.73</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CTNKH30831</t>
+          <t>IAFSA - NKJ0B80CKPKH34433</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -679,20 +679,20 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Cadereyta Jiménez</t>
+          <t>General Escobedo</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>34.41</v>
+        <v>330.45</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CHNKH30825</t>
+          <t>IAFSA - NKJ0B80CKNKH30816</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -717,20 +717,20 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Ciudad Santa Catarina</t>
+          <t>General Escobedo</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>23.23</v>
+        <v>247.41</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CTNKH30831</t>
+          <t>IAFSA - NKJ0B80CKNKH30816</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -755,20 +755,20 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Apodaca</t>
+          <t>Lampazos de Naranjo</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>18.59</v>
+        <v>194.98</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CTNKH30831</t>
+          <t>IAFSA - NKJ0B80CKPKH34433</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -788,21 +788,21 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Chihuahua</t>
+          <t>Nuevo León</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Chihuahua</t>
+          <t>Apodaca</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>9.31</v>
+        <v>189.04</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -831,20 +831,20 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>El Carmen</t>
+          <t>Monterrey</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>3.57</v>
+        <v>185.97</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CHNKH30825</t>
+          <t>IAFSA - NKJ0B80CKPKH34433</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -869,20 +869,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Guadalupe</t>
+          <t>Monterrey</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>3.07</v>
+        <v>170.86</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IAFSA - NKJ0B80CHNKH30825</t>
+          <t>IAFSA - NKJ0B80CKPKH34433</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -907,48 +907,656 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Monterrey</t>
+          <t>Cadereyta Jiménez</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>0.51</v>
+        <v>170.2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>IAFSA - NKJ0B80CKPKH34433</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>NEW HOLLAND CE</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>B80C</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Nuevo León</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>San Pedro Garza García</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>145.79</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>IAFSA - NKJ0B80CKNKH30816</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>NEW HOLLAND CE</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>B80C</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Nuevo León</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>San Pedro Garza García</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>138.63</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>IAFSA - NKJ0B80CTNKH30831</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>NEW HOLLAND CE</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>B80C</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Nuevo León</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>San Nicolás de los Garza</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>136.8</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>IAFSA - NKJ0B80CTNKH30831</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>NEW HOLLAND CE</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>B80C</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Nuevo León</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>San Pedro Garza García</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>108.41</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>IAFSA - NKJ0B80CKNKH30816</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>NEW HOLLAND CE</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>B80C</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Nuevo León</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Ciudad Santa Catarina</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>87.22</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>IAFSA - NKJ0B80CKPKH34433</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>NEW HOLLAND CE</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>B80C</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Nuevo León</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Guadalupe</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>64.38</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>IAFSA - NKJ0B80CTNKH30831</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>NEW HOLLAND CE</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>B80C</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Nuevo León</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Guadalupe</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>62.04</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>IAFSA - NKJ0B80CKPKH34433</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>NEW HOLLAND CE</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>B80C</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Nuevo León</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Ciudad Santa Catarina</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>58.98</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>IAFSA - NKJ0B80CHNKH30825</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>NEW HOLLAND CE</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>B80C</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Nuevo León</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>San Nicolás de los Garza</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>51.77</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>IAFSA - NKJ0B80CTNKH30831</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>NEW HOLLAND CE</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>B80C</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Nuevo León</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Cadereyta Jiménez</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>34.41</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>IAFSA - NKJ0B80CHNKH30825</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>NEW HOLLAND CE</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>B80C</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Nuevo León</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Ciudad Santa Catarina</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>23.23</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>IAFSA - NKJ0B80CTNKH30831</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>NEW HOLLAND CE</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>B80C</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Nuevo León</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Apodaca</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>18.59</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>IAFSA - NKJ0B80CTNKH30831</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>NEW HOLLAND CE</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>B80C</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Chihuahua</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Chihuahua</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>9.31</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>IAFSA - NKJ0B80CTNKH30831</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>NEW HOLLAND CE</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>B80C</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Nuevo León</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>El Carmen</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>3.57</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>IAFSA - NKJ0B80CHNKH30825</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>NEW HOLLAND CE</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>B80C</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Nuevo León</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Guadalupe</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>3.07</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>IAFSA - NKJ0B80CHNKH30825</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>NEW HOLLAND CE</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>B80C</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Nuevo León</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Monterrey</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
         <v>29</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>IAFSA - NKJ0B80CHNKH30825</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>NEW HOLLAND CE</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>B80C</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Nuevo León</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>INSUMOS AGROPECUARIOS FRONTERIZOS SA DE CV</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>NEW HOLLAND CE</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>B80C</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Nuevo León</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
         <is>
           <t>San Pedro Garza García</t>
         </is>
       </c>
-      <c r="H14" t="n">
+      <c r="H30" t="n">
         <v>0.04</v>
       </c>
     </row>

</xml_diff>